<commit_message>
Rewrite 31.08 order with the actual final numbers and exceptions
The first draft matched 30.08's text by mistake; the real order that
came in afterward has different counts (13/25 instead of 15/16) and a
different standard-block exception list (без говядины, без молочки
"сыр можно" + без тушеных овощей, instead of the previous carrot/pea/
rice combination).

Added two new composition categories this required: "говядина" (beef,
distinct from свинина/мясо) and "молочка_без_сыра" (dairy-except-cheese,
for "без молочки, сыр можно" - deliberately excludes сыр/фета/брынза/
рикотта/моцарелла from the tracked keywords, unlike the general
"лактоза" category).

Also replaced the earlier "КОТЛЕТА ДОМАШНЯЯ БЕЗ ЛУКА И БАТОНА" invented
variant with a real substitute (ГРУДКА КУРИНАЯ) - onion is mixed into
ground meat before cooking, so it can't actually be left out the way an
ingredient can be omitted from a garnish or salad.
</commit_message>
<xml_diff>
--- a/output/Гонконг 31.08.2026 (обработка).xlsx
+++ b/output/Гонконг 31.08.2026 (обработка).xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X62"/>
+  <dimension ref="A1:X59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.75" customWidth="1" min="1" max="1"/>
@@ -698,7 +698,7 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>БЕЗ БУЛГУРА И КИНОА</t>
+          <t>БЕЗ БУЛГАРА, БЕЗ КИНОА</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
@@ -733,32 +733,32 @@
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
+          <t>БЕЗ ГОВЯДИНЫ</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
           <t>БЕЗ КАШ</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>БЕЗ МОЛОЧКИ, БЕЗ ЛУКА, БЕЗ ГЛЮТЕНА, БЕЗ МОРКОВКИ, БЕЗ РИСА</t>
-        </is>
-      </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>БЕЗ СЫРОЙ МОРКОВИ, ГОРОХА, ЯБЛОК</t>
+          <t>БЕЗ РЫБЫ</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
+          <t>БЕЗ МОЛОЧКИ (СЫР МОЖНО), БЕЗ ТУШЕНЫХ ОВОЩЕЙ</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
           <t>БЕЗ РЫБЫ</t>
         </is>
       </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>БЕЗ РЫБЫ</t>
-        </is>
-      </c>
       <c r="W2" s="3" t="inlineStr">
         <is>
-          <t>БЕЗ САХАРА, РИСА И ПЕЧЕНИ</t>
+          <t>БЕЗ САХАРА, БЕЗ РИСА, БЕЗ ПЕЧЕНИ</t>
         </is>
       </c>
       <c r="X2" s="3" t="inlineStr"/>
@@ -912,10 +912,10 @@
         <v>1</v>
       </c>
       <c r="M4" s="9" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="O4" s="9" t="n">
         <v>3</v>
@@ -1114,16 +1114,16 @@
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R6" s="15" t="n"/>
+      <c r="R6" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
       <c r="S6" s="15" t="n"/>
       <c r="T6" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U6" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
+      <c r="U6" s="15" t="n"/>
       <c r="V6" s="15" t="n"/>
       <c r="W6" s="15" t="n"/>
       <c r="X6" s="15" t="n"/>
@@ -1160,12 +1160,12 @@
       </c>
       <c r="Q7" s="9" t="n"/>
       <c r="R7" s="9" t="n"/>
-      <c r="S7" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S7" s="9" t="n"/>
       <c r="T7" s="9" t="n"/>
-      <c r="U7" s="9" t="n"/>
+      <c r="U7" s="9">
+        <f>U4</f>
+        <v/>
+      </c>
       <c r="V7" s="9" t="n"/>
       <c r="W7" s="9" t="n"/>
       <c r="X7" s="9" t="n"/>
@@ -1274,15 +1274,15 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S9" s="15" t="n"/>
+      <c r="S9" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T9" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U9" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
+      <c r="U9" s="15" t="n"/>
       <c r="V9" s="15" t="n"/>
       <c r="W9" s="15" t="n"/>
       <c r="X9" s="15" t="n"/>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="Q10" s="9" t="n"/>
       <c r="R10" s="9" t="n"/>
-      <c r="S10" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S10" s="9" t="n"/>
       <c r="T10" s="9" t="n"/>
-      <c r="U10" s="9" t="n"/>
+      <c r="U10" s="9">
+        <f>U4</f>
+        <v/>
+      </c>
       <c r="V10" s="9">
         <f>V4</f>
         <v/>
@@ -1397,15 +1397,15 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S11" s="15" t="n"/>
+      <c r="S11" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T11" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U11" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
+      <c r="U11" s="15" t="n"/>
       <c r="V11" s="15">
         <f>V4</f>
         <v/>
@@ -1451,12 +1451,12 @@
       </c>
       <c r="Q12" s="9" t="n"/>
       <c r="R12" s="9" t="n"/>
-      <c r="S12" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S12" s="9" t="n"/>
       <c r="T12" s="9" t="n"/>
-      <c r="U12" s="9" t="n"/>
+      <c r="U12" s="9">
+        <f>U4</f>
+        <v/>
+      </c>
       <c r="V12" s="9" t="n"/>
       <c r="W12" s="9" t="n"/>
       <c r="X12" s="9" t="n"/>
@@ -1559,7 +1559,10 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S14" s="15" t="n"/>
+      <c r="S14" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T14" s="15">
         <f>T4</f>
         <v/>
@@ -1631,15 +1634,15 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S15" s="15" t="n"/>
+      <c r="S15" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T15" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U15" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
+      <c r="U15" s="15" t="n"/>
       <c r="V15" s="15">
         <f>V4</f>
         <v/>
@@ -2097,7 +2100,10 @@
         <f>S4</f>
         <v/>
       </c>
-      <c r="T20" s="15" t="n"/>
+      <c r="T20" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
       <c r="U20" s="15">
         <f>U4</f>
         <v/>
@@ -2116,622 +2122,685 @@
       </c>
     </row>
     <row r="21" ht="37.5" customHeight="1">
-      <c r="A21" s="1" t="n"/>
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t>ФРУКТЫ СВЕЖИЕ (БАНАН)</t>
-        </is>
-      </c>
-      <c r="C21" s="9">
+      <c r="A21" s="13" t="n"/>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>НАПИТОК</t>
+        </is>
+      </c>
+      <c r="C21" s="15">
         <f>SUM(D21:X21)</f>
         <v/>
       </c>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="9" t="n"/>
-      <c r="G21" s="9" t="n"/>
-      <c r="H21" s="9" t="n"/>
-      <c r="I21" s="9" t="n"/>
-      <c r="J21" s="9" t="n"/>
-      <c r="K21" s="9" t="n"/>
-      <c r="L21" s="9" t="n"/>
-      <c r="M21" s="9" t="n"/>
-      <c r="N21" s="9" t="n"/>
-      <c r="O21" s="9" t="n"/>
-      <c r="P21" s="9" t="n"/>
-      <c r="Q21" s="9" t="n"/>
-      <c r="R21" s="9" t="n"/>
-      <c r="S21" s="9" t="n"/>
-      <c r="T21" s="9">
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G21" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H21" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I21" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J21" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K21" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L21" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M21" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N21" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O21" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P21" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q21" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R21" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S21" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T21" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U21" s="9" t="n"/>
-      <c r="V21" s="9" t="n"/>
-      <c r="W21" s="9" t="n"/>
-      <c r="X21" s="9" t="n"/>
+      <c r="U21" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V21" s="15" t="n"/>
+      <c r="W21" s="15" t="n"/>
+      <c r="X21" s="15" t="n"/>
     </row>
     <row r="22" ht="37.5" customHeight="1">
-      <c r="A22" s="13" t="n"/>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>НАПИТОК</t>
-        </is>
-      </c>
-      <c r="C22" s="15">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>НАПИТОК БЕЗ САХАРА</t>
+        </is>
+      </c>
+      <c r="C22" s="9">
         <f>SUM(D22:X22)</f>
         <v/>
       </c>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="15">
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="9" t="n"/>
+      <c r="M22" s="9" t="n"/>
+      <c r="N22" s="9" t="n"/>
+      <c r="O22" s="9" t="n"/>
+      <c r="P22" s="9" t="n"/>
+      <c r="Q22" s="9" t="n"/>
+      <c r="R22" s="9" t="n"/>
+      <c r="S22" s="9" t="n"/>
+      <c r="T22" s="9" t="n"/>
+      <c r="U22" s="9" t="n"/>
+      <c r="V22" s="9">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W22" s="9">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X22" s="9">
+        <f>X4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="37.5" customHeight="1">
+      <c r="A23" s="13" t="n"/>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>БОУЛ С КУРИЦЕЙ ТЕРИЯКИ</t>
+        </is>
+      </c>
+      <c r="C23" s="15">
+        <f>SUM(D23:X23)</f>
+        <v/>
+      </c>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G22" s="15">
+      <c r="G23" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H22" s="15">
+      <c r="H23" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I22" s="15">
+      <c r="I23" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J22" s="15">
+      <c r="J23" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K22" s="15">
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M23" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N23" s="15" t="n"/>
+      <c r="O23" s="15" t="n"/>
+      <c r="P23" s="15" t="n"/>
+      <c r="Q23" s="15" t="n"/>
+      <c r="R23" s="15" t="n"/>
+      <c r="S23" s="15" t="n"/>
+      <c r="T23" s="15" t="n"/>
+      <c r="U23" s="15" t="n"/>
+      <c r="V23" s="15" t="n"/>
+      <c r="W23" s="15" t="n"/>
+      <c r="X23" s="15" t="n"/>
+    </row>
+    <row r="24" ht="37.5" customHeight="1">
+      <c r="A24" s="1" t="n"/>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>БОУЛ С КУРИЦЕЙ ТЕРИЯКИ БЕЗ КИНОА</t>
+        </is>
+      </c>
+      <c r="C24" s="9">
+        <f>SUM(D24:X24)</f>
+        <v/>
+      </c>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n"/>
+      <c r="I24" s="9" t="n"/>
+      <c r="J24" s="9" t="n"/>
+      <c r="K24" s="9">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L22" s="15">
+      <c r="L24" s="9" t="n"/>
+      <c r="M24" s="9" t="n"/>
+      <c r="N24" s="9" t="n"/>
+      <c r="O24" s="9" t="n"/>
+      <c r="P24" s="9" t="n"/>
+      <c r="Q24" s="9" t="n"/>
+      <c r="R24" s="9" t="n"/>
+      <c r="S24" s="9" t="n"/>
+      <c r="T24" s="9" t="n"/>
+      <c r="U24" s="9" t="n"/>
+      <c r="V24" s="9" t="n"/>
+      <c r="W24" s="9" t="n"/>
+      <c r="X24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="29.25" customHeight="1">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>ОБЕД</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="T25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="U25" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="V25" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="W25" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="X25" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="37.5" customHeight="1">
+      <c r="A26" s="13" t="n"/>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>САЛАТ ТЫКВЕННЫЙ С СЫРОМ</t>
+        </is>
+      </c>
+      <c r="C26" s="15">
+        <f>SUM(D26:X26)</f>
+        <v/>
+      </c>
+      <c r="D26" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E26" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H26" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I26" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J26" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K26" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L26" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M22" s="15">
+      <c r="M26" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N22" s="15">
+      <c r="N26" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O22" s="15">
+      <c r="O26" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P22" s="15">
+      <c r="P26" s="15" t="n"/>
+      <c r="Q26" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R26" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S26" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T26" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U26" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V26" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W26" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X26" s="15">
+        <f>X4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="37.5" customHeight="1">
+      <c r="A27" s="1" t="n"/>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>ОВОЩНОЙ САЛАТ</t>
+        </is>
+      </c>
+      <c r="C27" s="9">
+        <f>SUM(D27:X27)</f>
+        <v/>
+      </c>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="9" t="n"/>
+      <c r="F27" s="9">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="9" t="n"/>
+      <c r="I27" s="9" t="n"/>
+      <c r="J27" s="9" t="n"/>
+      <c r="K27" s="9" t="n"/>
+      <c r="L27" s="9" t="n"/>
+      <c r="M27" s="9" t="n"/>
+      <c r="N27" s="9" t="n"/>
+      <c r="O27" s="9" t="n"/>
+      <c r="P27" s="9">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q22" s="15">
+      <c r="Q27" s="9" t="n"/>
+      <c r="R27" s="9" t="n"/>
+      <c r="S27" s="9" t="n"/>
+      <c r="T27" s="9" t="n"/>
+      <c r="U27" s="9" t="n"/>
+      <c r="V27" s="9" t="n"/>
+      <c r="W27" s="9" t="n"/>
+      <c r="X27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="37.5" customHeight="1">
+      <c r="A28" s="13" t="n"/>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>БОРЩ С КУРИЦЕЙ</t>
+        </is>
+      </c>
+      <c r="C28" s="15">
+        <f>SUM(D28:X28)</f>
+        <v/>
+      </c>
+      <c r="D28" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E28" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="F28" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G28" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H28" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I28" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J28" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K28" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L28" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M28" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N28" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O28" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P28" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q28" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R22" s="15">
+      <c r="R28" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S22" s="15">
+      <c r="S28" s="15">
         <f>S4</f>
         <v/>
       </c>
-      <c r="T22" s="15">
+      <c r="T28" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U22" s="15">
+      <c r="U28" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V22" s="15" t="n"/>
-      <c r="W22" s="15" t="n"/>
-      <c r="X22" s="15" t="n"/>
-    </row>
-    <row r="23" ht="37.5" customHeight="1">
-      <c r="A23" s="1" t="n"/>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>НАПИТОК БЕЗ САХАРА</t>
-        </is>
-      </c>
-      <c r="C23" s="9">
-        <f>SUM(D23:X23)</f>
-        <v/>
-      </c>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="n"/>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="9" t="n"/>
-      <c r="H23" s="9" t="n"/>
-      <c r="I23" s="9" t="n"/>
-      <c r="J23" s="9" t="n"/>
-      <c r="K23" s="9" t="n"/>
-      <c r="L23" s="9" t="n"/>
-      <c r="M23" s="9" t="n"/>
-      <c r="N23" s="9" t="n"/>
-      <c r="O23" s="9" t="n"/>
-      <c r="P23" s="9" t="n"/>
-      <c r="Q23" s="9" t="n"/>
-      <c r="R23" s="9" t="n"/>
-      <c r="S23" s="9" t="n"/>
-      <c r="T23" s="9" t="n"/>
-      <c r="U23" s="9" t="n"/>
-      <c r="V23" s="9">
+      <c r="V28" s="15" t="n"/>
+      <c r="W28" s="15" t="n"/>
+      <c r="X28" s="15" t="n"/>
+    </row>
+    <row r="29" ht="37.5" customHeight="1">
+      <c r="A29" s="1" t="n"/>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>ТЫКВЕННЫЙ КРЕМ СУП</t>
+        </is>
+      </c>
+      <c r="C29" s="9">
+        <f>SUM(D29:X29)</f>
+        <v/>
+      </c>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="9" t="n"/>
+      <c r="I29" s="9" t="n"/>
+      <c r="J29" s="9" t="n"/>
+      <c r="K29" s="9" t="n"/>
+      <c r="L29" s="9" t="n"/>
+      <c r="M29" s="9" t="n"/>
+      <c r="N29" s="9" t="n"/>
+      <c r="O29" s="9" t="n"/>
+      <c r="P29" s="9" t="n"/>
+      <c r="Q29" s="9" t="n"/>
+      <c r="R29" s="9" t="n"/>
+      <c r="S29" s="9" t="n"/>
+      <c r="T29" s="9" t="n"/>
+      <c r="U29" s="9" t="n"/>
+      <c r="V29" s="9">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W23" s="9">
+      <c r="W29" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X23" s="9">
+      <c r="X29" s="9">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="37.5" customHeight="1">
-      <c r="A24" s="13" t="n"/>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>БОУЛ С КУРИЦЕЙ ТЕРИЯКИ</t>
-        </is>
-      </c>
-      <c r="C24" s="15">
-        <f>SUM(D24:X24)</f>
-        <v/>
-      </c>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15">
+    <row r="30" ht="37.5" customHeight="1">
+      <c r="A30" s="13" t="n"/>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>КОТЛЕТА ДОМАШНЯЯ</t>
+        </is>
+      </c>
+      <c r="C30" s="15">
+        <f>SUM(D30:X30)</f>
+        <v/>
+      </c>
+      <c r="D30" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E30" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="F30" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G24" s="15">
+      <c r="G30" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H24" s="15">
+      <c r="H30" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I24" s="15">
+      <c r="I30" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J24" s="15">
+      <c r="J30" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K24" s="15" t="n"/>
-      <c r="L24" s="15">
+      <c r="K30" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L30" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M24" s="15">
+      <c r="M30" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N24" s="15" t="n"/>
-      <c r="O24" s="15" t="n"/>
-      <c r="P24" s="15" t="n"/>
-      <c r="Q24" s="15" t="n"/>
-      <c r="R24" s="15" t="n"/>
-      <c r="S24" s="15" t="n"/>
-      <c r="T24" s="15" t="n"/>
-      <c r="U24" s="15" t="n"/>
-      <c r="V24" s="15" t="n"/>
-      <c r="W24" s="15" t="n"/>
-      <c r="X24" s="15" t="n"/>
-    </row>
-    <row r="25" ht="37.5" customHeight="1">
-      <c r="A25" s="1" t="n"/>
-      <c r="B25" s="16" t="inlineStr">
-        <is>
-          <t>БОУЛ С КУРИЦЕЙ ТЕРИЯКИ БЕЗ КИНОА</t>
-        </is>
-      </c>
-      <c r="C25" s="9">
-        <f>SUM(D25:X25)</f>
-        <v/>
-      </c>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="9" t="n"/>
-      <c r="H25" s="9" t="n"/>
-      <c r="I25" s="9" t="n"/>
-      <c r="J25" s="9" t="n"/>
-      <c r="K25" s="9">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L25" s="9" t="n"/>
-      <c r="M25" s="9" t="n"/>
-      <c r="N25" s="9" t="n"/>
-      <c r="O25" s="9" t="n"/>
-      <c r="P25" s="9" t="n"/>
-      <c r="Q25" s="9" t="n"/>
-      <c r="R25" s="9" t="n"/>
-      <c r="S25" s="9" t="n"/>
-      <c r="T25" s="9" t="n"/>
-      <c r="U25" s="9" t="n"/>
-      <c r="V25" s="9" t="n"/>
-      <c r="W25" s="9" t="n"/>
-      <c r="X25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="29.25" customHeight="1">
-      <c r="A26" s="10" t="n"/>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>ОБЕД</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="T26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="U26" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="V26" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="W26" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="X26" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="37.5" customHeight="1">
-      <c r="A27" s="13" t="n"/>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>САЛАТ ТЫКВЕННЫЙ С СЫРОМ</t>
-        </is>
-      </c>
-      <c r="C27" s="15">
-        <f>SUM(D27:X27)</f>
-        <v/>
-      </c>
-      <c r="D27" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E27" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H27" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I27" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J27" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K27" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L27" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M27" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N27" s="15">
+      <c r="N30" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O27" s="15">
+      <c r="O30" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P27" s="15" t="n"/>
-      <c r="Q27" s="15">
+      <c r="P30" s="15" t="n"/>
+      <c r="Q30" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R27" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S27" s="15" t="n"/>
-      <c r="T27" s="15">
+      <c r="R30" s="15" t="n"/>
+      <c r="S30" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T30" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U27" s="15">
+      <c r="U30" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V27" s="15">
+      <c r="V30" s="15">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W27" s="15">
+      <c r="W30" s="15">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X27" s="15">
+      <c r="X30" s="15">
         <f>X4</f>
         <v/>
       </c>
-    </row>
-    <row r="28" ht="37.5" customHeight="1">
-      <c r="A28" s="1" t="n"/>
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t>ОВОЩНОЙ САЛАТ</t>
-        </is>
-      </c>
-      <c r="C28" s="9">
-        <f>SUM(D28:X28)</f>
-        <v/>
-      </c>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="9">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G28" s="9" t="n"/>
-      <c r="H28" s="9" t="n"/>
-      <c r="I28" s="9" t="n"/>
-      <c r="J28" s="9" t="n"/>
-      <c r="K28" s="9" t="n"/>
-      <c r="L28" s="9" t="n"/>
-      <c r="M28" s="9" t="n"/>
-      <c r="N28" s="9" t="n"/>
-      <c r="O28" s="9" t="n"/>
-      <c r="P28" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q28" s="9" t="n"/>
-      <c r="R28" s="9" t="n"/>
-      <c r="S28" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T28" s="9" t="n"/>
-      <c r="U28" s="9" t="n"/>
-      <c r="V28" s="9" t="n"/>
-      <c r="W28" s="9" t="n"/>
-      <c r="X28" s="9" t="n"/>
-    </row>
-    <row r="29" ht="37.5" customHeight="1">
-      <c r="A29" s="13" t="n"/>
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>БОРЩ С КУРИЦЕЙ</t>
-        </is>
-      </c>
-      <c r="C29" s="15">
-        <f>SUM(D29:X29)</f>
-        <v/>
-      </c>
-      <c r="D29" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E29" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
-      <c r="F29" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G29" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H29" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I29" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J29" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K29" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L29" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M29" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N29" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O29" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P29" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q29" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R29" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S29" s="15" t="n"/>
-      <c r="T29" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U29" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V29" s="15" t="n"/>
-      <c r="W29" s="15" t="n"/>
-      <c r="X29" s="15" t="n"/>
-    </row>
-    <row r="30" ht="37.5" customHeight="1">
-      <c r="A30" s="1" t="n"/>
-      <c r="B30" s="16" t="inlineStr">
-        <is>
-          <t>БОРЩ С КУРИЦЕЙ БЕЗ ЛУКА И МОРКОВИ</t>
-        </is>
-      </c>
-      <c r="C30" s="9">
-        <f>SUM(D30:X30)</f>
-        <v/>
-      </c>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="9" t="n"/>
-      <c r="G30" s="9" t="n"/>
-      <c r="H30" s="9" t="n"/>
-      <c r="I30" s="9" t="n"/>
-      <c r="J30" s="9" t="n"/>
-      <c r="K30" s="9" t="n"/>
-      <c r="L30" s="9" t="n"/>
-      <c r="M30" s="9" t="n"/>
-      <c r="N30" s="9" t="n"/>
-      <c r="O30" s="9" t="n"/>
-      <c r="P30" s="9" t="n"/>
-      <c r="Q30" s="9" t="n"/>
-      <c r="R30" s="9" t="n"/>
-      <c r="S30" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T30" s="9" t="n"/>
-      <c r="U30" s="9" t="n"/>
-      <c r="V30" s="9" t="n"/>
-      <c r="W30" s="9" t="n"/>
-      <c r="X30" s="9" t="n"/>
     </row>
     <row r="31" ht="37.5" customHeight="1">
       <c r="A31" s="1" t="n"/>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>ТЫКВЕННЫЙ КРЕМ СУП</t>
+          <t>ГРУДКА КУРИНАЯ</t>
         </is>
       </c>
       <c r="C31" s="9">
@@ -2750,30 +2819,27 @@
       <c r="M31" s="9" t="n"/>
       <c r="N31" s="9" t="n"/>
       <c r="O31" s="9" t="n"/>
-      <c r="P31" s="9" t="n"/>
+      <c r="P31" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
       <c r="Q31" s="9" t="n"/>
-      <c r="R31" s="9" t="n"/>
+      <c r="R31" s="9">
+        <f>R4</f>
+        <v/>
+      </c>
       <c r="S31" s="9" t="n"/>
       <c r="T31" s="9" t="n"/>
       <c r="U31" s="9" t="n"/>
-      <c r="V31" s="9">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W31" s="9">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X31" s="9">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="V31" s="9" t="n"/>
+      <c r="W31" s="9" t="n"/>
+      <c r="X31" s="9" t="n"/>
     </row>
     <row r="32" ht="37.5" customHeight="1">
       <c r="A32" s="13" t="n"/>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>КОТЛЕТА ДОМАШНЯЯ</t>
+          <t>СПАГЕТТИ</t>
         </is>
       </c>
       <c r="C32" s="15">
@@ -2837,7 +2903,10 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S32" s="15" t="n"/>
+      <c r="S32" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T32" s="15">
         <f>T4</f>
         <v/>
@@ -2863,7 +2932,7 @@
       <c r="A33" s="1" t="n"/>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>КОТЛЕТА ДОМАШНЯЯ БЕЗ ЛУКА И БАТОНА</t>
+          <t>ОВОЩИ ЗАПЕЧЕННЫЕ</t>
         </is>
       </c>
       <c r="C33" s="9">
@@ -2888,10 +2957,7 @@
       </c>
       <c r="Q33" s="9" t="n"/>
       <c r="R33" s="9" t="n"/>
-      <c r="S33" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S33" s="9" t="n"/>
       <c r="T33" s="9" t="n"/>
       <c r="U33" s="9" t="n"/>
       <c r="V33" s="9" t="n"/>
@@ -2902,21 +2968,15 @@
       <c r="A34" s="13" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>СПАГЕТТИ</t>
+          <t>НАПИТОК</t>
         </is>
       </c>
       <c r="C34" s="15">
         <f>SUM(D34:X34)</f>
         <v/>
       </c>
-      <c r="D34" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E34" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
       <c r="F34" s="15">
         <f>F4</f>
         <v/>
@@ -2957,7 +3017,10 @@
         <f>O4</f>
         <v/>
       </c>
-      <c r="P34" s="15" t="n"/>
+      <c r="P34" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
       <c r="Q34" s="15">
         <f>Q4</f>
         <v/>
@@ -2966,7 +3029,10 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S34" s="15" t="n"/>
+      <c r="S34" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T34" s="15">
         <f>T4</f>
         <v/>
@@ -2975,24 +3041,15 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V34" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W34" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X34" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="V34" s="15" t="n"/>
+      <c r="W34" s="15" t="n"/>
+      <c r="X34" s="15" t="n"/>
     </row>
     <row r="35" ht="37.5" customHeight="1">
       <c r="A35" s="1" t="n"/>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>ОВОЩИ ЗАПЕЧЕННЫЕ</t>
+          <t>НАПИТОК БЕЗ САХАРА</t>
         </is>
       </c>
       <c r="C35" s="9">
@@ -3011,495 +3068,558 @@
       <c r="M35" s="9" t="n"/>
       <c r="N35" s="9" t="n"/>
       <c r="O35" s="9" t="n"/>
-      <c r="P35" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
+      <c r="P35" s="9" t="n"/>
       <c r="Q35" s="9" t="n"/>
       <c r="R35" s="9" t="n"/>
       <c r="S35" s="9" t="n"/>
       <c r="T35" s="9" t="n"/>
       <c r="U35" s="9" t="n"/>
-      <c r="V35" s="9" t="n"/>
-      <c r="W35" s="9" t="n"/>
-      <c r="X35" s="9" t="n"/>
+      <c r="V35" s="9">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W35" s="9">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X35" s="9">
+        <f>X4</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="37.5" customHeight="1">
-      <c r="A36" s="1" t="n"/>
-      <c r="B36" s="16" t="inlineStr">
-        <is>
-          <t>ОВОЩИ ЗАПЕЧЕННЫЕ БЕЗ МОРКОВИ</t>
-        </is>
-      </c>
-      <c r="C36" s="9">
+      <c r="A36" s="13" t="n"/>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
+        </is>
+      </c>
+      <c r="C36" s="15">
         <f>SUM(D36:X36)</f>
         <v/>
       </c>
-      <c r="D36" s="9" t="n"/>
-      <c r="E36" s="9" t="n"/>
-      <c r="F36" s="9" t="n"/>
-      <c r="G36" s="9" t="n"/>
-      <c r="H36" s="9" t="n"/>
-      <c r="I36" s="9" t="n"/>
-      <c r="J36" s="9" t="n"/>
-      <c r="K36" s="9" t="n"/>
-      <c r="L36" s="9" t="n"/>
-      <c r="M36" s="9" t="n"/>
-      <c r="N36" s="9" t="n"/>
-      <c r="O36" s="9" t="n"/>
-      <c r="P36" s="9" t="n"/>
-      <c r="Q36" s="9" t="n"/>
-      <c r="R36" s="9" t="n"/>
-      <c r="S36" s="9">
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="15" t="n"/>
+      <c r="F36" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G36" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H36" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I36" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J36" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K36" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L36" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M36" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N36" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O36" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P36" s="15" t="n"/>
+      <c r="Q36" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R36" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S36" s="15">
         <f>S4</f>
         <v/>
       </c>
-      <c r="T36" s="9" t="n"/>
-      <c r="U36" s="9" t="n"/>
-      <c r="V36" s="9" t="n"/>
-      <c r="W36" s="9" t="n"/>
-      <c r="X36" s="9" t="n"/>
-    </row>
-    <row r="37" ht="37.5" customHeight="1">
-      <c r="A37" s="13" t="n"/>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="T36" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U36" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V36" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W36" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X36" s="15">
+        <f>X4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="29.25" customHeight="1">
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>ПОЛДНИК</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="T37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="U37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="V37" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="W37" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="X37" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="37.5" customHeight="1">
+      <c r="A38" s="13" t="n"/>
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>НАПИТОК</t>
         </is>
       </c>
-      <c r="C37" s="15">
-        <f>SUM(D37:X37)</f>
-        <v/>
-      </c>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="15" t="n"/>
-      <c r="F37" s="15">
+      <c r="C38" s="15">
+        <f>SUM(D38:X38)</f>
+        <v/>
+      </c>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="15" t="n"/>
+      <c r="F38" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G37" s="15">
+      <c r="G38" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H37" s="15">
+      <c r="H38" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I37" s="15">
+      <c r="I38" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J37" s="15">
+      <c r="J38" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K37" s="15">
+      <c r="K38" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L37" s="15">
+      <c r="L38" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M37" s="15">
+      <c r="M38" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N37" s="15">
+      <c r="N38" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O37" s="15">
+      <c r="O38" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P37" s="15">
+      <c r="P38" s="15">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q37" s="15">
+      <c r="Q38" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R37" s="15">
+      <c r="R38" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S37" s="15">
+      <c r="S38" s="15">
         <f>S4</f>
         <v/>
       </c>
-      <c r="T37" s="15">
+      <c r="T38" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U37" s="15">
+      <c r="U38" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V37" s="15" t="n"/>
-      <c r="W37" s="15" t="n"/>
-      <c r="X37" s="15" t="n"/>
-    </row>
-    <row r="38" ht="37.5" customHeight="1">
-      <c r="A38" s="1" t="n"/>
-      <c r="B38" s="16" t="inlineStr">
+      <c r="V38" s="15" t="n"/>
+      <c r="W38" s="15" t="n"/>
+      <c r="X38" s="15" t="n"/>
+    </row>
+    <row r="39" ht="37.5" customHeight="1">
+      <c r="A39" s="1" t="n"/>
+      <c r="B39" s="16" t="inlineStr">
         <is>
           <t>НАПИТОК БЕЗ САХАРА</t>
         </is>
       </c>
-      <c r="C38" s="9">
-        <f>SUM(D38:X38)</f>
-        <v/>
-      </c>
-      <c r="D38" s="9" t="n"/>
-      <c r="E38" s="9" t="n"/>
-      <c r="F38" s="9" t="n"/>
-      <c r="G38" s="9" t="n"/>
-      <c r="H38" s="9" t="n"/>
-      <c r="I38" s="9" t="n"/>
-      <c r="J38" s="9" t="n"/>
-      <c r="K38" s="9" t="n"/>
-      <c r="L38" s="9" t="n"/>
-      <c r="M38" s="9" t="n"/>
-      <c r="N38" s="9" t="n"/>
-      <c r="O38" s="9" t="n"/>
-      <c r="P38" s="9" t="n"/>
-      <c r="Q38" s="9" t="n"/>
-      <c r="R38" s="9" t="n"/>
-      <c r="S38" s="9" t="n"/>
-      <c r="T38" s="9" t="n"/>
-      <c r="U38" s="9" t="n"/>
-      <c r="V38" s="9">
+      <c r="C39" s="9">
+        <f>SUM(D39:X39)</f>
+        <v/>
+      </c>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" s="9" t="n"/>
+      <c r="J39" s="9" t="n"/>
+      <c r="K39" s="9" t="n"/>
+      <c r="L39" s="9" t="n"/>
+      <c r="M39" s="9" t="n"/>
+      <c r="N39" s="9" t="n"/>
+      <c r="O39" s="9" t="n"/>
+      <c r="P39" s="9" t="n"/>
+      <c r="Q39" s="9" t="n"/>
+      <c r="R39" s="9" t="n"/>
+      <c r="S39" s="9" t="n"/>
+      <c r="T39" s="9" t="n"/>
+      <c r="U39" s="9" t="n"/>
+      <c r="V39" s="9">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W38" s="9">
+      <c r="W39" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X38" s="9">
+      <c r="X39" s="9">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="39" ht="37.5" customHeight="1">
-      <c r="A39" s="13" t="n"/>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
-        </is>
-      </c>
-      <c r="C39" s="15">
-        <f>SUM(D39:X39)</f>
-        <v/>
-      </c>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="15" t="n"/>
-      <c r="F39" s="15">
+    <row r="40" ht="37.5" customHeight="1">
+      <c r="A40" s="13" t="n"/>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ПЕЧЕНЬЕ </t>
+        </is>
+      </c>
+      <c r="C40" s="15">
+        <f>SUM(D40:X40)</f>
+        <v/>
+      </c>
+      <c r="D40" s="15" t="n"/>
+      <c r="E40" s="15" t="n"/>
+      <c r="F40" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G39" s="15">
+      <c r="G40" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H39" s="15">
+      <c r="H40" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I39" s="15">
+      <c r="I40" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J39" s="15">
+      <c r="J40" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K39" s="15">
+      <c r="K40" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L39" s="15">
+      <c r="L40" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M39" s="15">
+      <c r="M40" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N39" s="15">
+      <c r="N40" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O39" s="15">
+      <c r="O40" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P39" s="15" t="n"/>
-      <c r="Q39" s="15">
+      <c r="P40" s="15" t="n"/>
+      <c r="Q40" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R39" s="15">
+      <c r="R40" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S39" s="15" t="n"/>
-      <c r="T39" s="15">
+      <c r="S40" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T40" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U39" s="15">
+      <c r="U40" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V39" s="15">
+      <c r="V40" s="15" t="n"/>
+      <c r="W40" s="15" t="n"/>
+      <c r="X40" s="15" t="n"/>
+    </row>
+    <row r="41" ht="37.5" customHeight="1">
+      <c r="A41" s="1" t="n"/>
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>ЯБЛОКО ЗАПЕЧЕННОЕ</t>
+        </is>
+      </c>
+      <c r="C41" s="9">
+        <f>SUM(D41:X41)</f>
+        <v/>
+      </c>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="9" t="n"/>
+      <c r="F41" s="9" t="n"/>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9" t="n"/>
+      <c r="I41" s="9" t="n"/>
+      <c r="J41" s="9" t="n"/>
+      <c r="K41" s="9" t="n"/>
+      <c r="L41" s="9" t="n"/>
+      <c r="M41" s="9" t="n"/>
+      <c r="N41" s="9" t="n"/>
+      <c r="O41" s="9" t="n"/>
+      <c r="P41" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q41" s="9" t="n"/>
+      <c r="R41" s="9" t="n"/>
+      <c r="S41" s="9" t="n"/>
+      <c r="T41" s="9" t="n"/>
+      <c r="U41" s="9" t="n"/>
+      <c r="V41" s="9">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W39" s="15">
+      <c r="W41" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X39" s="15">
+      <c r="X41" s="9">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="40" ht="29.25" customHeight="1">
-      <c r="A40" s="10" t="n"/>
-      <c r="B40" s="11" t="inlineStr">
-        <is>
-          <t>ПОЛДНИК</t>
-        </is>
-      </c>
-      <c r="C40" s="10" t="n"/>
-      <c r="D40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="T40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="U40" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="V40" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="W40" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="X40" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="37.5" customHeight="1">
-      <c r="A41" s="13" t="n"/>
-      <c r="B41" s="14" t="inlineStr">
-        <is>
-          <t>НАПИТОК</t>
-        </is>
-      </c>
-      <c r="C41" s="15">
-        <f>SUM(D41:X41)</f>
-        <v/>
-      </c>
-      <c r="D41" s="15" t="n"/>
-      <c r="E41" s="15" t="n"/>
-      <c r="F41" s="15">
+    <row r="42" ht="37.5" customHeight="1">
+      <c r="A42" s="13" t="n"/>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>ЧАЙ</t>
+        </is>
+      </c>
+      <c r="C42" s="15">
+        <f>SUM(D42:X42)</f>
+        <v/>
+      </c>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G41" s="15">
+      <c r="G42" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H41" s="15">
+      <c r="H42" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I41" s="15">
+      <c r="I42" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J41" s="15">
+      <c r="J42" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K41" s="15">
+      <c r="K42" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L41" s="15">
+      <c r="L42" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M41" s="15">
+      <c r="M42" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N41" s="15">
+      <c r="N42" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O41" s="15">
+      <c r="O42" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P41" s="15">
+      <c r="P42" s="15">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q41" s="15">
+      <c r="Q42" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R41" s="15">
+      <c r="R42" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S41" s="15">
+      <c r="S42" s="15">
         <f>S4</f>
         <v/>
       </c>
-      <c r="T41" s="15">
+      <c r="T42" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U41" s="15">
+      <c r="U42" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V41" s="15" t="n"/>
-      <c r="W41" s="15" t="n"/>
-      <c r="X41" s="15" t="n"/>
-    </row>
-    <row r="42" ht="37.5" customHeight="1">
-      <c r="A42" s="1" t="n"/>
-      <c r="B42" s="16" t="inlineStr">
-        <is>
-          <t>НАПИТОК БЕЗ САХАРА</t>
-        </is>
-      </c>
-      <c r="C42" s="9">
-        <f>SUM(D42:X42)</f>
-        <v/>
-      </c>
-      <c r="D42" s="9" t="n"/>
-      <c r="E42" s="9" t="n"/>
-      <c r="F42" s="9" t="n"/>
-      <c r="G42" s="9" t="n"/>
-      <c r="H42" s="9" t="n"/>
-      <c r="I42" s="9" t="n"/>
-      <c r="J42" s="9" t="n"/>
-      <c r="K42" s="9" t="n"/>
-      <c r="L42" s="9" t="n"/>
-      <c r="M42" s="9" t="n"/>
-      <c r="N42" s="9" t="n"/>
-      <c r="O42" s="9" t="n"/>
-      <c r="P42" s="9" t="n"/>
-      <c r="Q42" s="9" t="n"/>
-      <c r="R42" s="9" t="n"/>
-      <c r="S42" s="9" t="n"/>
-      <c r="T42" s="9" t="n"/>
-      <c r="U42" s="9" t="n"/>
-      <c r="V42" s="9">
+      <c r="V42" s="15">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W42" s="9">
+      <c r="W42" s="15">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X42" s="9">
+      <c r="X42" s="15">
         <f>X4</f>
         <v/>
       </c>
@@ -3508,7 +3628,7 @@
       <c r="A43" s="13" t="n"/>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">ПЕЧЕНЬЕ </t>
+          <t>САХАР ПОРЦИОННЫЙ</t>
         </is>
       </c>
       <c r="C43" s="15">
@@ -3557,7 +3677,10 @@
         <f>O4</f>
         <v/>
       </c>
-      <c r="P43" s="15" t="n"/>
+      <c r="P43" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
       <c r="Q43" s="15">
         <f>Q4</f>
         <v/>
@@ -3566,7 +3689,10 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S43" s="15" t="n"/>
+      <c r="S43" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T43" s="15">
         <f>T4</f>
         <v/>
@@ -3579,67 +3705,139 @@
       <c r="W43" s="15" t="n"/>
       <c r="X43" s="15" t="n"/>
     </row>
-    <row r="44" ht="37.5" customHeight="1">
-      <c r="A44" s="1" t="n"/>
-      <c r="B44" s="16" t="inlineStr">
-        <is>
-          <t>ЯБЛОКО ЗАПЕЧЕННОЕ</t>
-        </is>
-      </c>
-      <c r="C44" s="9">
-        <f>SUM(D44:X44)</f>
-        <v/>
-      </c>
-      <c r="D44" s="9" t="n"/>
-      <c r="E44" s="9" t="n"/>
-      <c r="F44" s="9" t="n"/>
-      <c r="G44" s="9" t="n"/>
-      <c r="H44" s="9" t="n"/>
-      <c r="I44" s="9" t="n"/>
-      <c r="J44" s="9" t="n"/>
-      <c r="K44" s="9" t="n"/>
-      <c r="L44" s="9" t="n"/>
-      <c r="M44" s="9" t="n"/>
-      <c r="N44" s="9" t="n"/>
-      <c r="O44" s="9" t="n"/>
-      <c r="P44" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q44" s="9" t="n"/>
-      <c r="R44" s="9" t="n"/>
-      <c r="S44" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T44" s="9" t="n"/>
-      <c r="U44" s="9" t="n"/>
-      <c r="V44" s="9">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W44" s="9">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X44" s="9">
-        <f>X4</f>
-        <v/>
+    <row r="44" ht="29.25" customHeight="1">
+      <c r="A44" s="10" t="n"/>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>УЖИН</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="T44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="U44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="V44" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="W44" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="X44" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
       </c>
     </row>
     <row r="45" ht="37.5" customHeight="1">
       <c r="A45" s="13" t="n"/>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>ЧАЙ</t>
+          <t>САЛАТ С КИНОА И БУЛГУРОМ</t>
         </is>
       </c>
       <c r="C45" s="15">
         <f>SUM(D45:X45)</f>
         <v/>
       </c>
-      <c r="D45" s="15" t="n"/>
-      <c r="E45" s="15" t="n"/>
+      <c r="D45" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E45" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
       <c r="F45" s="15">
         <f>F4</f>
         <v/>
@@ -3660,10 +3858,7 @@
         <f>J4</f>
         <v/>
       </c>
-      <c r="K45" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
+      <c r="K45" s="15" t="n"/>
       <c r="L45" s="15">
         <f>L4</f>
         <v/>
@@ -3680,10 +3875,7 @@
         <f>O4</f>
         <v/>
       </c>
-      <c r="P45" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
+      <c r="P45" s="15" t="n"/>
       <c r="Q45" s="15">
         <f>Q4</f>
         <v/>
@@ -3718,292 +3910,160 @@
       </c>
     </row>
     <row r="46" ht="37.5" customHeight="1">
-      <c r="A46" s="13" t="n"/>
-      <c r="B46" s="14" t="inlineStr">
-        <is>
-          <t>САХАР ПОРЦИОННЫЙ</t>
-        </is>
-      </c>
-      <c r="C46" s="15">
+      <c r="A46" s="1" t="n"/>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>САЛАТ ЗЕЛЕНЫЙ С КУКУРУЗОЙ</t>
+        </is>
+      </c>
+      <c r="C46" s="9">
         <f>SUM(D46:X46)</f>
         <v/>
       </c>
-      <c r="D46" s="15" t="n"/>
-      <c r="E46" s="15" t="n"/>
-      <c r="F46" s="15">
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="F46" s="9" t="n"/>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="9" t="n"/>
+      <c r="I46" s="9" t="n"/>
+      <c r="J46" s="9" t="n"/>
+      <c r="K46" s="9">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L46" s="9" t="n"/>
+      <c r="M46" s="9" t="n"/>
+      <c r="N46" s="9" t="n"/>
+      <c r="O46" s="9" t="n"/>
+      <c r="P46" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q46" s="9" t="n"/>
+      <c r="R46" s="9" t="n"/>
+      <c r="S46" s="9" t="n"/>
+      <c r="T46" s="9" t="n"/>
+      <c r="U46" s="9" t="n"/>
+      <c r="V46" s="9" t="n"/>
+      <c r="W46" s="9" t="n"/>
+      <c r="X46" s="9" t="n"/>
+    </row>
+    <row r="47" ht="37.5" customHeight="1">
+      <c r="A47" s="13" t="n"/>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>ТРЕСКА С КОПЧЕНЫМ БАТАТОМ</t>
+        </is>
+      </c>
+      <c r="C47" s="15">
+        <f>SUM(D47:X47)</f>
+        <v/>
+      </c>
+      <c r="D47" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E47" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="F47" s="15" t="n"/>
+      <c r="G47" s="15" t="n"/>
+      <c r="H47" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I47" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J47" s="15" t="n"/>
+      <c r="K47" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L47" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M47" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N47" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O47" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P47" s="15" t="n"/>
+      <c r="Q47" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R47" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S47" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T47" s="15" t="n"/>
+      <c r="U47" s="15" t="n"/>
+      <c r="V47" s="15" t="n"/>
+      <c r="W47" s="15" t="n"/>
+      <c r="X47" s="15" t="n"/>
+    </row>
+    <row r="48" ht="37.5" customHeight="1">
+      <c r="A48" s="1" t="n"/>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>ТРЕСКА С КОПЧЕНЫМ БАТАТОМ БЕЗ ЛАКТОЗЫ</t>
+        </is>
+      </c>
+      <c r="C48" s="9">
+        <f>SUM(D48:X48)</f>
+        <v/>
+      </c>
+      <c r="D48" s="9" t="n"/>
+      <c r="E48" s="9" t="n"/>
+      <c r="F48" s="9">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G46" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H46" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I46" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J46" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K46" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L46" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M46" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N46" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O46" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P46" s="15">
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n"/>
+      <c r="I48" s="9" t="n"/>
+      <c r="J48" s="9" t="n"/>
+      <c r="K48" s="9" t="n"/>
+      <c r="L48" s="9" t="n"/>
+      <c r="M48" s="9" t="n"/>
+      <c r="N48" s="9" t="n"/>
+      <c r="O48" s="9" t="n"/>
+      <c r="P48" s="9">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q46" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R46" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S46" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T46" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U46" s="15">
+      <c r="Q48" s="9" t="n"/>
+      <c r="R48" s="9" t="n"/>
+      <c r="S48" s="9" t="n"/>
+      <c r="T48" s="9" t="n"/>
+      <c r="U48" s="9">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V46" s="15" t="n"/>
-      <c r="W46" s="15" t="n"/>
-      <c r="X46" s="15" t="n"/>
-    </row>
-    <row r="47" ht="29.25" customHeight="1">
-      <c r="A47" s="10" t="n"/>
-      <c r="B47" s="11" t="inlineStr">
-        <is>
-          <t>УЖИН</t>
-        </is>
-      </c>
-      <c r="C47" s="10" t="n"/>
-      <c r="D47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="T47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="U47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="V47" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="W47" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="X47" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="37.5" customHeight="1">
-      <c r="A48" s="13" t="n"/>
-      <c r="B48" s="14" t="inlineStr">
-        <is>
-          <t>САЛАТ С КИНОА И БУЛГУРОМ</t>
-        </is>
-      </c>
-      <c r="C48" s="15">
-        <f>SUM(D48:X48)</f>
-        <v/>
-      </c>
-      <c r="D48" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E48" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
-      <c r="F48" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G48" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H48" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I48" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J48" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K48" s="15" t="n"/>
-      <c r="L48" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M48" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N48" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O48" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P48" s="15" t="n"/>
-      <c r="Q48" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R48" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S48" s="15" t="n"/>
-      <c r="T48" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U48" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V48" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W48" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X48" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="V48" s="9" t="n"/>
+      <c r="W48" s="9" t="n"/>
+      <c r="X48" s="9" t="n"/>
     </row>
     <row r="49" ht="37.5" customHeight="1">
       <c r="A49" s="1" t="n"/>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>САЛАТ ЗЕЛЕНЫЙ С КУКУРУЗОЙ</t>
+          <t>ТРЕСКА С КОПЧЕНЫМ БАТАТОМ БЕЗ БАТАТА</t>
         </is>
       </c>
       <c r="C49" s="9">
@@ -4017,146 +4077,161 @@
       <c r="H49" s="9" t="n"/>
       <c r="I49" s="9" t="n"/>
       <c r="J49" s="9" t="n"/>
-      <c r="K49" s="9">
-        <f>K4</f>
-        <v/>
-      </c>
+      <c r="K49" s="9" t="n"/>
       <c r="L49" s="9" t="n"/>
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="9" t="n"/>
       <c r="O49" s="9" t="n"/>
-      <c r="P49" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
+      <c r="P49" s="9" t="n"/>
       <c r="Q49" s="9" t="n"/>
       <c r="R49" s="9" t="n"/>
-      <c r="S49" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S49" s="9" t="n"/>
       <c r="T49" s="9" t="n"/>
       <c r="U49" s="9" t="n"/>
       <c r="V49" s="9" t="n"/>
-      <c r="W49" s="9" t="n"/>
-      <c r="X49" s="9" t="n"/>
+      <c r="W49" s="9">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X49" s="9">
+        <f>X4</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="37.5" customHeight="1">
-      <c r="A50" s="13" t="n"/>
-      <c r="B50" s="14" t="inlineStr">
-        <is>
-          <t>ТРЕСКА С КОПЧЕНЫМ БАТАТОМ</t>
-        </is>
-      </c>
-      <c r="C50" s="15">
+      <c r="A50" s="1" t="n"/>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>ИНДЕЙКА ГРУДКА</t>
+        </is>
+      </c>
+      <c r="C50" s="9">
         <f>SUM(D50:X50)</f>
         <v/>
       </c>
-      <c r="D50" s="15">
+      <c r="D50" s="9" t="n"/>
+      <c r="E50" s="9" t="n"/>
+      <c r="F50" s="9" t="n"/>
+      <c r="G50" s="9">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H50" s="9" t="n"/>
+      <c r="I50" s="9" t="n"/>
+      <c r="J50" s="9">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K50" s="9" t="n"/>
+      <c r="L50" s="9" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="9" t="n"/>
+      <c r="O50" s="9" t="n"/>
+      <c r="P50" s="9" t="n"/>
+      <c r="Q50" s="9" t="n"/>
+      <c r="R50" s="9" t="n"/>
+      <c r="S50" s="9" t="n"/>
+      <c r="T50" s="9">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U50" s="9" t="n"/>
+      <c r="V50" s="9">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W50" s="9" t="n"/>
+      <c r="X50" s="9" t="n"/>
+    </row>
+    <row r="51" ht="37.5" customHeight="1">
+      <c r="A51" s="13" t="n"/>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>РИС ОТВАРНОЙ С ЗЕЛЕНЬЮ И СЛИВОЧНЫМ МАСЛОМ</t>
+        </is>
+      </c>
+      <c r="C51" s="15">
+        <f>SUM(D51:X51)</f>
+        <v/>
+      </c>
+      <c r="D51" s="15">
         <f>D4</f>
         <v/>
       </c>
-      <c r="E50" s="15">
+      <c r="E51" s="15">
         <f>E4</f>
         <v/>
       </c>
-      <c r="F50" s="15" t="n"/>
-      <c r="G50" s="15" t="n"/>
-      <c r="H50" s="15">
+      <c r="F51" s="15" t="n"/>
+      <c r="G51" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H51" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I50" s="15">
+      <c r="I51" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J50" s="15" t="n"/>
-      <c r="K50" s="15">
+      <c r="J51" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K51" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L50" s="15">
+      <c r="L51" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M50" s="15">
+      <c r="M51" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N50" s="15">
+      <c r="N51" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O50" s="15">
+      <c r="O51" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P50" s="15" t="n"/>
-      <c r="Q50" s="15">
+      <c r="P51" s="15" t="n"/>
+      <c r="Q51" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R50" s="15">
+      <c r="R51" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S50" s="15" t="n"/>
-      <c r="T50" s="15">
+      <c r="S51" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T51" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U50" s="15" t="n"/>
-      <c r="V50" s="15" t="n"/>
-      <c r="W50" s="15" t="n"/>
-      <c r="X50" s="15" t="n"/>
-    </row>
-    <row r="51" ht="37.5" customHeight="1">
-      <c r="A51" s="1" t="n"/>
-      <c r="B51" s="16" t="inlineStr">
-        <is>
-          <t>ТРЕСКА С КОПЧЕНЫМ БАТАТОМ БЕЗ ЛАКТОЗЫ</t>
-        </is>
-      </c>
-      <c r="C51" s="9">
-        <f>SUM(D51:X51)</f>
-        <v/>
-      </c>
-      <c r="D51" s="9" t="n"/>
-      <c r="E51" s="9" t="n"/>
-      <c r="F51" s="9">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G51" s="9" t="n"/>
-      <c r="H51" s="9" t="n"/>
-      <c r="I51" s="9" t="n"/>
-      <c r="J51" s="9" t="n"/>
-      <c r="K51" s="9" t="n"/>
-      <c r="L51" s="9" t="n"/>
-      <c r="M51" s="9" t="n"/>
-      <c r="N51" s="9" t="n"/>
-      <c r="O51" s="9" t="n"/>
-      <c r="P51" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q51" s="9" t="n"/>
-      <c r="R51" s="9" t="n"/>
-      <c r="S51" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T51" s="9" t="n"/>
-      <c r="U51" s="9" t="n"/>
-      <c r="V51" s="9" t="n"/>
-      <c r="W51" s="9" t="n"/>
-      <c r="X51" s="9" t="n"/>
+      <c r="U51" s="15" t="n"/>
+      <c r="V51" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W51" s="15" t="n"/>
+      <c r="X51" s="15">
+        <f>X4</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="37.5" customHeight="1">
       <c r="A52" s="1" t="n"/>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>ИНДЕЙКА ГРУДКА</t>
+          <t>РИС ОТВАРНОЙ С ЗЕЛЕНЬЮ БЕЗ СЛИВОЧНОГО МАСЛА</t>
         </is>
       </c>
       <c r="C52" s="9">
@@ -4165,23 +4240,23 @@
       </c>
       <c r="D52" s="9" t="n"/>
       <c r="E52" s="9" t="n"/>
-      <c r="F52" s="9" t="n"/>
-      <c r="G52" s="9">
-        <f>G4</f>
-        <v/>
-      </c>
+      <c r="F52" s="9">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G52" s="9" t="n"/>
       <c r="H52" s="9" t="n"/>
       <c r="I52" s="9" t="n"/>
-      <c r="J52" s="9">
-        <f>J4</f>
-        <v/>
-      </c>
+      <c r="J52" s="9" t="n"/>
       <c r="K52" s="9" t="n"/>
       <c r="L52" s="9" t="n"/>
       <c r="M52" s="9" t="n"/>
       <c r="N52" s="9" t="n"/>
       <c r="O52" s="9" t="n"/>
-      <c r="P52" s="9" t="n"/>
+      <c r="P52" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
       <c r="Q52" s="9" t="n"/>
       <c r="R52" s="9" t="n"/>
       <c r="S52" s="9" t="n"/>
@@ -4190,309 +4265,423 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V52" s="9">
+      <c r="V52" s="9" t="n"/>
+      <c r="W52" s="9" t="n"/>
+      <c r="X52" s="9" t="n"/>
+    </row>
+    <row r="53" ht="37.5" customHeight="1">
+      <c r="A53" s="1" t="n"/>
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>КУС КУС С ОВОЩАМИ</t>
+        </is>
+      </c>
+      <c r="C53" s="9">
+        <f>SUM(D53:X53)</f>
+        <v/>
+      </c>
+      <c r="D53" s="9" t="n"/>
+      <c r="E53" s="9" t="n"/>
+      <c r="F53" s="9" t="n"/>
+      <c r="G53" s="9" t="n"/>
+      <c r="H53" s="9" t="n"/>
+      <c r="I53" s="9" t="n"/>
+      <c r="J53" s="9" t="n"/>
+      <c r="K53" s="9" t="n"/>
+      <c r="L53" s="9" t="n"/>
+      <c r="M53" s="9" t="n"/>
+      <c r="N53" s="9" t="n"/>
+      <c r="O53" s="9" t="n"/>
+      <c r="P53" s="9" t="n"/>
+      <c r="Q53" s="9" t="n"/>
+      <c r="R53" s="9" t="n"/>
+      <c r="S53" s="9" t="n"/>
+      <c r="T53" s="9" t="n"/>
+      <c r="U53" s="9" t="n"/>
+      <c r="V53" s="9" t="n"/>
+      <c r="W53" s="9">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X53" s="9" t="n"/>
+    </row>
+    <row r="54" ht="37.5" customHeight="1">
+      <c r="A54" s="13" t="n"/>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>ЧАЙ</t>
+        </is>
+      </c>
+      <c r="C54" s="15">
+        <f>SUM(D54:X54)</f>
+        <v/>
+      </c>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="15" t="n"/>
+      <c r="F54" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G54" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H54" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I54" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J54" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K54" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L54" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M54" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N54" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O54" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P54" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q54" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R54" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S54" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T54" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U54" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V54" s="15">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W52" s="9">
+      <c r="W54" s="15">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X52" s="9">
+      <c r="X54" s="15">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="53" ht="37.5" customHeight="1">
-      <c r="A53" s="13" t="n"/>
-      <c r="B53" s="14" t="inlineStr">
-        <is>
-          <t>РИС ОТВАРНОЙ С ЗЕЛЕНЬЮ И СЛИВОЧНЫМ МАСЛОМ</t>
-        </is>
-      </c>
-      <c r="C53" s="15">
-        <f>SUM(D53:X53)</f>
-        <v/>
-      </c>
-      <c r="D53" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E53" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
-      <c r="F53" s="15" t="n"/>
-      <c r="G53" s="15">
+    <row r="55" ht="37.5" customHeight="1">
+      <c r="A55" s="13" t="n"/>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>САХАР ПОРЦИОННЫЙ</t>
+        </is>
+      </c>
+      <c r="C55" s="15">
+        <f>SUM(D55:X55)</f>
+        <v/>
+      </c>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="15" t="n"/>
+      <c r="F55" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G55" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H53" s="15">
+      <c r="H55" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I53" s="15">
+      <c r="I55" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J53" s="15">
+      <c r="J55" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K53" s="15">
+      <c r="K55" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L53" s="15">
+      <c r="L55" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M53" s="15">
+      <c r="M55" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N53" s="15">
+      <c r="N55" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O53" s="15">
+      <c r="O55" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P53" s="15" t="n"/>
-      <c r="Q53" s="15">
+      <c r="P55" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q55" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R53" s="15">
+      <c r="R55" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S53" s="15" t="n"/>
-      <c r="T53" s="15">
+      <c r="S55" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T55" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U53" s="15">
+      <c r="U55" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V53" s="15">
+      <c r="V55" s="15" t="n"/>
+      <c r="W55" s="15" t="n"/>
+      <c r="X55" s="15" t="n"/>
+    </row>
+    <row r="56" ht="37.5" customHeight="1">
+      <c r="A56" s="13" t="n"/>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
+        </is>
+      </c>
+      <c r="C56" s="15">
+        <f>SUM(D56:X56)</f>
+        <v/>
+      </c>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="15" t="n"/>
+      <c r="F56" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G56" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H56" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I56" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J56" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K56" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L56" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M56" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N56" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O56" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P56" s="15" t="n"/>
+      <c r="Q56" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R56" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S56" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T56" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U56" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V56" s="15">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W53" s="15" t="n"/>
-      <c r="X53" s="15">
+      <c r="W56" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X56" s="15">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="54" ht="37.5" customHeight="1">
-      <c r="A54" s="1" t="n"/>
-      <c r="B54" s="16" t="inlineStr">
-        <is>
-          <t>РИС ОТВАРНОЙ С ЗЕЛЕНЬЮ БЕЗ СЛИВОЧНОГО МАСЛА</t>
-        </is>
-      </c>
-      <c r="C54" s="9">
-        <f>SUM(D54:X54)</f>
-        <v/>
-      </c>
-      <c r="D54" s="9" t="n"/>
-      <c r="E54" s="9" t="n"/>
-      <c r="F54" s="9">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G54" s="9" t="n"/>
-      <c r="H54" s="9" t="n"/>
-      <c r="I54" s="9" t="n"/>
-      <c r="J54" s="9" t="n"/>
-      <c r="K54" s="9" t="n"/>
-      <c r="L54" s="9" t="n"/>
-      <c r="M54" s="9" t="n"/>
-      <c r="N54" s="9" t="n"/>
-      <c r="O54" s="9" t="n"/>
-      <c r="P54" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q54" s="9" t="n"/>
-      <c r="R54" s="9" t="n"/>
-      <c r="S54" s="9" t="n"/>
-      <c r="T54" s="9" t="n"/>
-      <c r="U54" s="9" t="n"/>
-      <c r="V54" s="9" t="n"/>
-      <c r="W54" s="9" t="n"/>
-      <c r="X54" s="9" t="n"/>
-    </row>
-    <row r="55" ht="37.5" customHeight="1">
-      <c r="A55" s="1" t="n"/>
-      <c r="B55" s="16" t="inlineStr">
-        <is>
-          <t>КАРТОФЕЛЬ ЗАПЕЧЕННЫЙ</t>
-        </is>
-      </c>
-      <c r="C55" s="9">
-        <f>SUM(D55:X55)</f>
-        <v/>
-      </c>
-      <c r="D55" s="9" t="n"/>
-      <c r="E55" s="9" t="n"/>
-      <c r="F55" s="9" t="n"/>
-      <c r="G55" s="9" t="n"/>
-      <c r="H55" s="9" t="n"/>
-      <c r="I55" s="9" t="n"/>
-      <c r="J55" s="9" t="n"/>
-      <c r="K55" s="9" t="n"/>
-      <c r="L55" s="9" t="n"/>
-      <c r="M55" s="9" t="n"/>
-      <c r="N55" s="9" t="n"/>
-      <c r="O55" s="9" t="n"/>
-      <c r="P55" s="9" t="n"/>
-      <c r="Q55" s="9" t="n"/>
-      <c r="R55" s="9" t="n"/>
-      <c r="S55" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T55" s="9" t="n"/>
-      <c r="U55" s="9" t="n"/>
-      <c r="V55" s="9" t="n"/>
-      <c r="W55" s="9" t="n"/>
-      <c r="X55" s="9" t="n"/>
-    </row>
-    <row r="56" ht="37.5" customHeight="1">
-      <c r="A56" s="1" t="n"/>
-      <c r="B56" s="16" t="inlineStr">
-        <is>
-          <t>КУС КУС С ОВОЩАМИ</t>
-        </is>
-      </c>
-      <c r="C56" s="9">
-        <f>SUM(D56:X56)</f>
-        <v/>
-      </c>
-      <c r="D56" s="9" t="n"/>
-      <c r="E56" s="9" t="n"/>
-      <c r="F56" s="9" t="n"/>
-      <c r="G56" s="9" t="n"/>
-      <c r="H56" s="9" t="n"/>
-      <c r="I56" s="9" t="n"/>
-      <c r="J56" s="9" t="n"/>
-      <c r="K56" s="9" t="n"/>
-      <c r="L56" s="9" t="n"/>
-      <c r="M56" s="9" t="n"/>
-      <c r="N56" s="9" t="n"/>
-      <c r="O56" s="9" t="n"/>
-      <c r="P56" s="9" t="n"/>
-      <c r="Q56" s="9" t="n"/>
-      <c r="R56" s="9" t="n"/>
-      <c r="S56" s="9" t="n"/>
-      <c r="T56" s="9" t="n"/>
-      <c r="U56" s="9" t="n"/>
-      <c r="V56" s="9" t="n"/>
-      <c r="W56" s="9">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X56" s="9" t="n"/>
-    </row>
-    <row r="57" ht="37.5" customHeight="1">
-      <c r="A57" s="13" t="n"/>
-      <c r="B57" s="14" t="inlineStr">
-        <is>
-          <t>ЧАЙ</t>
-        </is>
-      </c>
-      <c r="C57" s="15">
-        <f>SUM(D57:X57)</f>
-        <v/>
-      </c>
-      <c r="D57" s="15" t="n"/>
-      <c r="E57" s="15" t="n"/>
-      <c r="F57" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G57" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H57" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I57" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J57" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K57" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L57" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M57" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N57" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O57" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P57" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q57" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R57" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S57" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T57" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U57" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V57" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W57" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X57" s="15">
-        <f>X4</f>
-        <v/>
+    <row r="57" ht="29.25" customHeight="1">
+      <c r="A57" s="10" t="n"/>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>2-Й УЖИН</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="n"/>
+      <c r="D57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="T57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="U57" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="V57" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="W57" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="X57" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
       </c>
     </row>
     <row r="58" ht="37.5" customHeight="1">
       <c r="A58" s="13" t="n"/>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>САХАР ПОРЦИОННЫЙ</t>
+          <t>КЕФИР</t>
         </is>
       </c>
       <c r="C58" s="15">
@@ -4501,10 +4690,7 @@
       </c>
       <c r="D58" s="15" t="n"/>
       <c r="E58" s="15" t="n"/>
-      <c r="F58" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
+      <c r="F58" s="15" t="n"/>
       <c r="G58" s="15">
         <f>G4</f>
         <v/>
@@ -4541,10 +4727,7 @@
         <f>O4</f>
         <v/>
       </c>
-      <c r="P58" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
+      <c r="P58" s="15" t="n"/>
       <c r="Q58" s="15">
         <f>Q4</f>
         <v/>
@@ -4561,334 +4744,61 @@
         <f>T4</f>
         <v/>
       </c>
-      <c r="U58" s="15">
+      <c r="U58" s="15" t="n"/>
+      <c r="V58" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W58" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X58" s="15">
+        <f>X4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="37.5" customHeight="1">
+      <c r="A59" s="1" t="n"/>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>НАПИТОК</t>
+        </is>
+      </c>
+      <c r="C59" s="9">
+        <f>SUM(D59:X59)</f>
+        <v/>
+      </c>
+      <c r="D59" s="9" t="n"/>
+      <c r="E59" s="9" t="n"/>
+      <c r="F59" s="9">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G59" s="9" t="n"/>
+      <c r="H59" s="9" t="n"/>
+      <c r="I59" s="9" t="n"/>
+      <c r="J59" s="9" t="n"/>
+      <c r="K59" s="9" t="n"/>
+      <c r="L59" s="9" t="n"/>
+      <c r="M59" s="9" t="n"/>
+      <c r="N59" s="9" t="n"/>
+      <c r="O59" s="9" t="n"/>
+      <c r="P59" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q59" s="9" t="n"/>
+      <c r="R59" s="9" t="n"/>
+      <c r="S59" s="9" t="n"/>
+      <c r="T59" s="9" t="n"/>
+      <c r="U59" s="9">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V58" s="15" t="n"/>
-      <c r="W58" s="15" t="n"/>
-      <c r="X58" s="15" t="n"/>
-    </row>
-    <row r="59" ht="37.5" customHeight="1">
-      <c r="A59" s="13" t="n"/>
-      <c r="B59" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
-        </is>
-      </c>
-      <c r="C59" s="15">
-        <f>SUM(D59:X59)</f>
-        <v/>
-      </c>
-      <c r="D59" s="15" t="n"/>
-      <c r="E59" s="15" t="n"/>
-      <c r="F59" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G59" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H59" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I59" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J59" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K59" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L59" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M59" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N59" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O59" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P59" s="15" t="n"/>
-      <c r="Q59" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R59" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S59" s="15" t="n"/>
-      <c r="T59" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U59" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V59" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W59" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X59" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="29.25" customHeight="1">
-      <c r="A60" s="10" t="n"/>
-      <c r="B60" s="11" t="inlineStr">
-        <is>
-          <t>2-Й УЖИН</t>
-        </is>
-      </c>
-      <c r="C60" s="10" t="n"/>
-      <c r="D60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="T60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="U60" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="V60" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="W60" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="X60" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="37.5" customHeight="1">
-      <c r="A61" s="13" t="n"/>
-      <c r="B61" s="14" t="inlineStr">
-        <is>
-          <t>КЕФИР</t>
-        </is>
-      </c>
-      <c r="C61" s="15">
-        <f>SUM(D61:X61)</f>
-        <v/>
-      </c>
-      <c r="D61" s="15" t="n"/>
-      <c r="E61" s="15" t="n"/>
-      <c r="F61" s="15" t="n"/>
-      <c r="G61" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H61" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I61" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J61" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K61" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L61" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M61" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N61" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O61" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P61" s="15" t="n"/>
-      <c r="Q61" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R61" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S61" s="15" t="n"/>
-      <c r="T61" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U61" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V61" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W61" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X61" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="37.5" customHeight="1">
-      <c r="A62" s="1" t="n"/>
-      <c r="B62" s="16" t="inlineStr">
-        <is>
-          <t>НАПИТОК</t>
-        </is>
-      </c>
-      <c r="C62" s="9">
-        <f>SUM(D62:X62)</f>
-        <v/>
-      </c>
-      <c r="D62" s="9" t="n"/>
-      <c r="E62" s="9" t="n"/>
-      <c r="F62" s="9">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G62" s="9" t="n"/>
-      <c r="H62" s="9" t="n"/>
-      <c r="I62" s="9" t="n"/>
-      <c r="J62" s="9" t="n"/>
-      <c r="K62" s="9" t="n"/>
-      <c r="L62" s="9" t="n"/>
-      <c r="M62" s="9" t="n"/>
-      <c r="N62" s="9" t="n"/>
-      <c r="O62" s="9" t="n"/>
-      <c r="P62" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q62" s="9" t="n"/>
-      <c r="R62" s="9" t="n"/>
-      <c r="S62" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T62" s="9" t="n"/>
-      <c r="U62" s="9" t="n"/>
-      <c r="V62" s="9" t="n"/>
-      <c r="W62" s="9" t="n"/>
-      <c r="X62" s="9" t="n"/>
+      <c r="V59" s="9" t="n"/>
+      <c r="W59" s="9" t="n"/>
+      <c r="X59" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Merge treska's two dinner alternatives into one (sauce is the batata)
The lactose and the potato exclusions on this dish are the same
component - the sauce is made from batata (milk/cream + sweet potato).
Removing the sauce entirely satisfies both at once, so F/P/U (lactose)
and W/X (potato) - 7 people total - now get a single "без соуса" plain
cod instead of two separately-fabricated variants.
</commit_message>
<xml_diff>
--- a/output/Гонконг 31.08.2026 (обработка).xlsx
+++ b/output/Гонконг 31.08.2026 (обработка).xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X58"/>
+  <dimension ref="A1:X57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.75" customWidth="1" min="1" max="1"/>
@@ -3988,7 +3988,7 @@
       <c r="A47" s="1" t="n"/>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>ТРЕСКА С КОПЧЕНЫМ БАТАТОМ БЕЗ ЛАКТОЗЫ</t>
+          <t>ТРЕСКА БЕЗ СОУСА</t>
         </is>
       </c>
       <c r="C47" s="9">
@@ -4023,14 +4023,20 @@
         <v/>
       </c>
       <c r="V47" s="9" t="n"/>
-      <c r="W47" s="9" t="n"/>
-      <c r="X47" s="9" t="n"/>
+      <c r="W47" s="9">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X47" s="9">
+        <f>X4</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="37.5" customHeight="1">
       <c r="A48" s="1" t="n"/>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>ТРЕСКА С КОПЧЕНЫМ БАТАТОМ БЕЗ БАТАТА</t>
+          <t>ИНДЕЙКА ГРУДКА</t>
         </is>
       </c>
       <c r="C48" s="9">
@@ -4040,10 +4046,16 @@
       <c r="D48" s="9" t="n"/>
       <c r="E48" s="9" t="n"/>
       <c r="F48" s="9" t="n"/>
-      <c r="G48" s="9" t="n"/>
+      <c r="G48" s="9">
+        <f>G4</f>
+        <v/>
+      </c>
       <c r="H48" s="9" t="n"/>
       <c r="I48" s="9" t="n"/>
-      <c r="J48" s="9" t="n"/>
+      <c r="J48" s="9">
+        <f>J4</f>
+        <v/>
+      </c>
       <c r="K48" s="9" t="n"/>
       <c r="L48" s="9" t="n"/>
       <c r="M48" s="9" t="n"/>
@@ -4053,152 +4065,149 @@
       <c r="Q48" s="9" t="n"/>
       <c r="R48" s="9" t="n"/>
       <c r="S48" s="9" t="n"/>
-      <c r="T48" s="9" t="n"/>
+      <c r="T48" s="9">
+        <f>T4</f>
+        <v/>
+      </c>
       <c r="U48" s="9" t="n"/>
-      <c r="V48" s="9" t="n"/>
-      <c r="W48" s="9">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X48" s="9">
+      <c r="V48" s="9">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W48" s="9" t="n"/>
+      <c r="X48" s="9" t="n"/>
+    </row>
+    <row r="49" ht="37.5" customHeight="1">
+      <c r="A49" s="13" t="n"/>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>РИС ОТВАРНОЙ С ЗЕЛЕНЬЮ И СЛИВОЧНЫМ МАСЛОМ</t>
+        </is>
+      </c>
+      <c r="C49" s="15">
+        <f>SUM(D49:X49)</f>
+        <v/>
+      </c>
+      <c r="D49" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E49" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="F49" s="15" t="n"/>
+      <c r="G49" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H49" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I49" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J49" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K49" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L49" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M49" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N49" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O49" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P49" s="15" t="n"/>
+      <c r="Q49" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R49" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S49" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T49" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U49" s="15" t="n"/>
+      <c r="V49" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W49" s="15" t="n"/>
+      <c r="X49" s="15">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="49" ht="37.5" customHeight="1">
-      <c r="A49" s="1" t="n"/>
-      <c r="B49" s="16" t="inlineStr">
-        <is>
-          <t>ИНДЕЙКА ГРУДКА</t>
-        </is>
-      </c>
-      <c r="C49" s="9">
-        <f>SUM(D49:X49)</f>
-        <v/>
-      </c>
-      <c r="D49" s="9" t="n"/>
-      <c r="E49" s="9" t="n"/>
-      <c r="F49" s="9" t="n"/>
-      <c r="G49" s="9">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H49" s="9" t="n"/>
-      <c r="I49" s="9" t="n"/>
-      <c r="J49" s="9">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K49" s="9" t="n"/>
-      <c r="L49" s="9" t="n"/>
-      <c r="M49" s="9" t="n"/>
-      <c r="N49" s="9" t="n"/>
-      <c r="O49" s="9" t="n"/>
-      <c r="P49" s="9" t="n"/>
-      <c r="Q49" s="9" t="n"/>
-      <c r="R49" s="9" t="n"/>
-      <c r="S49" s="9" t="n"/>
-      <c r="T49" s="9">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U49" s="9" t="n"/>
-      <c r="V49" s="9">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W49" s="9" t="n"/>
-      <c r="X49" s="9" t="n"/>
-    </row>
     <row r="50" ht="37.5" customHeight="1">
-      <c r="A50" s="13" t="n"/>
-      <c r="B50" s="14" t="inlineStr">
-        <is>
-          <t>РИС ОТВАРНОЙ С ЗЕЛЕНЬЮ И СЛИВОЧНЫМ МАСЛОМ</t>
-        </is>
-      </c>
-      <c r="C50" s="15">
+      <c r="A50" s="1" t="n"/>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>РИС ОТВАРНОЙ С ЗЕЛЕНЬЮ БЕЗ СЛИВОЧНОГО МАСЛА</t>
+        </is>
+      </c>
+      <c r="C50" s="9">
         <f>SUM(D50:X50)</f>
         <v/>
       </c>
-      <c r="D50" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E50" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
-      <c r="F50" s="15" t="n"/>
-      <c r="G50" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H50" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I50" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J50" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K50" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L50" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M50" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N50" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O50" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P50" s="15" t="n"/>
-      <c r="Q50" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R50" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S50" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T50" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U50" s="15" t="n"/>
-      <c r="V50" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W50" s="15" t="n"/>
-      <c r="X50" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="D50" s="9" t="n"/>
+      <c r="E50" s="9" t="n"/>
+      <c r="F50" s="9">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G50" s="9" t="n"/>
+      <c r="H50" s="9" t="n"/>
+      <c r="I50" s="9" t="n"/>
+      <c r="J50" s="9" t="n"/>
+      <c r="K50" s="9" t="n"/>
+      <c r="L50" s="9" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="9" t="n"/>
+      <c r="O50" s="9" t="n"/>
+      <c r="P50" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q50" s="9" t="n"/>
+      <c r="R50" s="9" t="n"/>
+      <c r="S50" s="9" t="n"/>
+      <c r="T50" s="9" t="n"/>
+      <c r="U50" s="9">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V50" s="9" t="n"/>
+      <c r="W50" s="9" t="n"/>
+      <c r="X50" s="9" t="n"/>
     </row>
     <row r="51" ht="37.5" customHeight="1">
       <c r="A51" s="1" t="n"/>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>РИС ОТВАРНОЙ С ЗЕЛЕНЬЮ БЕЗ СЛИВОЧНОГО МАСЛА</t>
+          <t>КУС КУС С ОВОЩАМИ</t>
         </is>
       </c>
       <c r="C51" s="9">
@@ -4207,10 +4216,7 @@
       </c>
       <c r="D51" s="9" t="n"/>
       <c r="E51" s="9" t="n"/>
-      <c r="F51" s="9">
-        <f>F4</f>
-        <v/>
-      </c>
+      <c r="F51" s="9" t="n"/>
       <c r="G51" s="9" t="n"/>
       <c r="H51" s="9" t="n"/>
       <c r="I51" s="9" t="n"/>
@@ -4220,63 +4226,114 @@
       <c r="M51" s="9" t="n"/>
       <c r="N51" s="9" t="n"/>
       <c r="O51" s="9" t="n"/>
-      <c r="P51" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
+      <c r="P51" s="9" t="n"/>
       <c r="Q51" s="9" t="n"/>
       <c r="R51" s="9" t="n"/>
       <c r="S51" s="9" t="n"/>
       <c r="T51" s="9" t="n"/>
-      <c r="U51" s="9">
+      <c r="U51" s="9" t="n"/>
+      <c r="V51" s="9" t="n"/>
+      <c r="W51" s="9">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X51" s="9" t="n"/>
+    </row>
+    <row r="52" ht="37.5" customHeight="1">
+      <c r="A52" s="13" t="n"/>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>ЧАЙ</t>
+        </is>
+      </c>
+      <c r="C52" s="15">
+        <f>SUM(D52:X52)</f>
+        <v/>
+      </c>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="15" t="n"/>
+      <c r="F52" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G52" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H52" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I52" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J52" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K52" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L52" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M52" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N52" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O52" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P52" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q52" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R52" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S52" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T52" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U52" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V51" s="9" t="n"/>
-      <c r="W51" s="9" t="n"/>
-      <c r="X51" s="9" t="n"/>
-    </row>
-    <row r="52" ht="37.5" customHeight="1">
-      <c r="A52" s="1" t="n"/>
-      <c r="B52" s="16" t="inlineStr">
-        <is>
-          <t>КУС КУС С ОВОЩАМИ</t>
-        </is>
-      </c>
-      <c r="C52" s="9">
-        <f>SUM(D52:X52)</f>
-        <v/>
-      </c>
-      <c r="D52" s="9" t="n"/>
-      <c r="E52" s="9" t="n"/>
-      <c r="F52" s="9" t="n"/>
-      <c r="G52" s="9" t="n"/>
-      <c r="H52" s="9" t="n"/>
-      <c r="I52" s="9" t="n"/>
-      <c r="J52" s="9" t="n"/>
-      <c r="K52" s="9" t="n"/>
-      <c r="L52" s="9" t="n"/>
-      <c r="M52" s="9" t="n"/>
-      <c r="N52" s="9" t="n"/>
-      <c r="O52" s="9" t="n"/>
-      <c r="P52" s="9" t="n"/>
-      <c r="Q52" s="9" t="n"/>
-      <c r="R52" s="9" t="n"/>
-      <c r="S52" s="9" t="n"/>
-      <c r="T52" s="9" t="n"/>
-      <c r="U52" s="9" t="n"/>
-      <c r="V52" s="9" t="n"/>
-      <c r="W52" s="9">
+      <c r="V52" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W52" s="15">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X52" s="9" t="n"/>
+      <c r="X52" s="15">
+        <f>X4</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="37.5" customHeight="1">
       <c r="A53" s="13" t="n"/>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>ЧАЙ</t>
+          <t>САХАР ПОРЦИОННЫЙ</t>
         </is>
       </c>
       <c r="C53" s="15">
@@ -4349,24 +4406,15 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V53" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W53" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X53" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="V53" s="15" t="n"/>
+      <c r="W53" s="15" t="n"/>
+      <c r="X53" s="15" t="n"/>
     </row>
     <row r="54" ht="37.5" customHeight="1">
       <c r="A54" s="13" t="n"/>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>САХАР ПОРЦИОННЫЙ</t>
+          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
         </is>
       </c>
       <c r="C54" s="15">
@@ -4415,10 +4463,7 @@
         <f>O4</f>
         <v/>
       </c>
-      <c r="P54" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
+      <c r="P54" s="15" t="n"/>
       <c r="Q54" s="15">
         <f>Q4</f>
         <v/>
@@ -4439,333 +4484,255 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V54" s="15" t="n"/>
-      <c r="W54" s="15" t="n"/>
-      <c r="X54" s="15" t="n"/>
-    </row>
-    <row r="55" ht="37.5" customHeight="1">
-      <c r="A55" s="13" t="n"/>
-      <c r="B55" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
-        </is>
-      </c>
-      <c r="C55" s="15">
-        <f>SUM(D55:X55)</f>
-        <v/>
-      </c>
-      <c r="D55" s="15" t="n"/>
-      <c r="E55" s="15" t="n"/>
-      <c r="F55" s="15">
+      <c r="V54" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W54" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X54" s="15">
+        <f>X4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="29.25" customHeight="1">
+      <c r="A55" s="10" t="n"/>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>2-Й УЖИН</t>
+        </is>
+      </c>
+      <c r="C55" s="10" t="n"/>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="T55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="U55" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="V55" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="W55" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="X55" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="37.5" customHeight="1">
+      <c r="A56" s="13" t="n"/>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>КЕФИР</t>
+        </is>
+      </c>
+      <c r="C56" s="15">
+        <f>SUM(D56:X56)</f>
+        <v/>
+      </c>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="15" t="n"/>
+      <c r="F56" s="15" t="n"/>
+      <c r="G56" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H56" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I56" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J56" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K56" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L56" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M56" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N56" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O56" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P56" s="15" t="n"/>
+      <c r="Q56" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R56" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S56" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T56" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U56" s="15" t="n"/>
+      <c r="V56" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W56" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X56" s="15">
+        <f>X4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="37.5" customHeight="1">
+      <c r="A57" s="1" t="n"/>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>НАПИТОК</t>
+        </is>
+      </c>
+      <c r="C57" s="9">
+        <f>SUM(D57:X57)</f>
+        <v/>
+      </c>
+      <c r="D57" s="9" t="n"/>
+      <c r="E57" s="9" t="n"/>
+      <c r="F57" s="9">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G55" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H55" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I55" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J55" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K55" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L55" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M55" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N55" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O55" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P55" s="15" t="n"/>
-      <c r="Q55" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R55" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S55" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T55" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U55" s="15">
+      <c r="G57" s="9" t="n"/>
+      <c r="H57" s="9" t="n"/>
+      <c r="I57" s="9" t="n"/>
+      <c r="J57" s="9" t="n"/>
+      <c r="K57" s="9" t="n"/>
+      <c r="L57" s="9" t="n"/>
+      <c r="M57" s="9" t="n"/>
+      <c r="N57" s="9" t="n"/>
+      <c r="O57" s="9" t="n"/>
+      <c r="P57" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q57" s="9" t="n"/>
+      <c r="R57" s="9" t="n"/>
+      <c r="S57" s="9" t="n"/>
+      <c r="T57" s="9" t="n"/>
+      <c r="U57" s="9">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V55" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W55" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X55" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" ht="29.25" customHeight="1">
-      <c r="A56" s="10" t="n"/>
-      <c r="B56" s="11" t="inlineStr">
-        <is>
-          <t>2-Й УЖИН</t>
-        </is>
-      </c>
-      <c r="C56" s="10" t="n"/>
-      <c r="D56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="T56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="U56" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="V56" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="W56" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="X56" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="37.5" customHeight="1">
-      <c r="A57" s="13" t="n"/>
-      <c r="B57" s="14" t="inlineStr">
-        <is>
-          <t>КЕФИР</t>
-        </is>
-      </c>
-      <c r="C57" s="15">
-        <f>SUM(D57:X57)</f>
-        <v/>
-      </c>
-      <c r="D57" s="15" t="n"/>
-      <c r="E57" s="15" t="n"/>
-      <c r="F57" s="15" t="n"/>
-      <c r="G57" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H57" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I57" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J57" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K57" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L57" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M57" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N57" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O57" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P57" s="15" t="n"/>
-      <c r="Q57" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R57" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S57" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T57" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U57" s="15" t="n"/>
-      <c r="V57" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W57" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X57" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" ht="37.5" customHeight="1">
-      <c r="A58" s="1" t="n"/>
-      <c r="B58" s="16" t="inlineStr">
-        <is>
-          <t>НАПИТОК</t>
-        </is>
-      </c>
-      <c r="C58" s="9">
-        <f>SUM(D58:X58)</f>
-        <v/>
-      </c>
-      <c r="D58" s="9" t="n"/>
-      <c r="E58" s="9" t="n"/>
-      <c r="F58" s="9">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G58" s="9" t="n"/>
-      <c r="H58" s="9" t="n"/>
-      <c r="I58" s="9" t="n"/>
-      <c r="J58" s="9" t="n"/>
-      <c r="K58" s="9" t="n"/>
-      <c r="L58" s="9" t="n"/>
-      <c r="M58" s="9" t="n"/>
-      <c r="N58" s="9" t="n"/>
-      <c r="O58" s="9" t="n"/>
-      <c r="P58" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q58" s="9" t="n"/>
-      <c r="R58" s="9" t="n"/>
-      <c r="S58" s="9" t="n"/>
-      <c r="T58" s="9" t="n"/>
-      <c r="U58" s="9">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V58" s="9" t="n"/>
-      <c r="W58" s="9" t="n"/>
-      <c r="X58" s="9" t="n"/>
+      <c r="V57" s="9" t="n"/>
+      <c r="W57" s="9" t="n"/>
+      <c r="X57" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>